<commit_message>
feat: add ai consensus adjudication workbook
</commit_message>
<xml_diff>
--- a/outputs/cf01_annotation_20260728/track_a_ai_comparison_review.xlsx
+++ b/outputs/cf01_annotation_20260728/track_a_ai_comparison_review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一致性摘要" sheetId="1" r:id="Rb9d1dc3b971d485b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心分歧审查" sheetId="2" r:id="Rf0a5b10c19cd41e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI逐题对比" sheetId="3" r:id="R0aab98560dd141a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI-A原始" sheetId="4" r:id="Radaad8662b54456e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI-B原始" sheetId="5" r:id="R28bfc8d3f9ae4a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一致性摘要" sheetId="1" r:id="R4fd39782ba2f4ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心分歧审查" sheetId="2" r:id="R4d39ec24d2794f3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI逐题对比" sheetId="3" r:id="Rbeb1a0b1ef264e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI-A原始" sheetId="4" r:id="Rafa5f7e993ad4b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI-B原始" sheetId="5" r:id="Re96e85ab4fce40f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +49,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,12 +73,17 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF2CC"/>
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF0F6B6D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -208,13 +213,13 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -375,7 +380,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Codex" id="{D60BC20D-90AD-4713-9C9A-8D1DD79D8B5B}"/>
+  <xltc:person displayName="Codex" id="{8B2D1A30-1A8E-4C1F-997C-82C9D3F61436}"/>
 </xltc:personList>
 </file>
 
@@ -794,7 +799,7 @@
         <x:v>AI-B元数据</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>缺失</x:v>
+        <x:v>完整</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
         <x:v>能力状态</x:v>
@@ -900,7 +905,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B16" s="38" t="str">
-        <x:v>AI-B原始文件缺少模型、时间和角色元数据，正式归档前应补齐。</x:v>
+        <x:v>AI-A模型记录为deepseek-v4-pro；AI-B模型身份已补录。时间字段不作为本轮AI辅助试标门槛。</x:v>
       </x:c>
       <x:c r="C16" s="38" t="str"/>
       <x:c r="D16" s="38" t="str"/>
@@ -1468,7 +1473,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab6bb70ad1a14a1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0960666618c24674"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3250,7 +3255,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29b682d48d3b4ac9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a36479d114948dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4104,7 +4109,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4520aae59e104b8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R702bdae74bd84dde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4958,7 +4963,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R921f168c7ac54b32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71d65dfc0d784224"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>